<commit_message>
RECEIVE: 300 ai pc in bhiwandi branch (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,6 +503,42 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ai pc</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>bhiwandi branch</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F3" t="n">
+        <v>300</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -519,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,6 +662,56 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>[{"batch_id": 1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-31T05:42:19.997942+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300 ai pc in bhiwandi branch</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ai pc</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>bhiwandi branch</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>300</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 2}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DISPATCH: sold 300 ai pc (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -495,7 +495,7 @@
         <v>300</v>
       </c>
       <c r="F2" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -712,6 +712,56 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>[{"batch_id": 2}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-31T05:42:42.106284+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sold 300 ai pc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ai pc</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>bhiwandi branch</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 1, "date_received": "2025-05-14", "qty_taken": 300}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log rejected message (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -762,6 +762,39 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>[{"batch_id": 1, "date_received": "2025-05-14", "qty_taken": 300}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-31T06:34:36.640406+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>we have 50 laptops from january 22 2026 in delhi</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>[]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RECEIVE: we have 50 laptops from january 22 2026 in delhi (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,6 +539,42 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>laptops</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>delhi</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -555,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -877,7 +913,6 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>krish</t>
@@ -891,6 +926,56 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-31T06:40:18.659814+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>we have 50 laptops from january 22 2026 in delhi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>laptops</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>delhi</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 3}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DISPATCH: sold 30 ai pc from bhiwandi (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -531,7 +531,7 @@
         <v>300</v>
       </c>
       <c r="F3" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -979,6 +979,56 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-31T06:53:26.983811+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sold 30 ai pc from bhiwandi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ai pc</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>bhiwandi branch</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 2, "date_received": "2026-07-31", "qty_taken": 30}]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>